<commit_message>
solving the problem about three cols
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -413,95 +413,162 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Shiva</t>
-        </is>
-      </c>
-      <c r="B1" t="n">
-        <v>25</v>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Shiva</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>HYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Ravi</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B3" t="n">
         <v>30</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>WGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="n">
         <v>28</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Kumar</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>22</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KZJ</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Kumar</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>22</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>HNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>Meena</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>27</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>HNK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="n">
         <v>35</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Arjun</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>29</v>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Arjun</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>WGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Sneha</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B9" t="n">
         <v>24</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SEC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="n">
         <v>31</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>HYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Kavya</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
         <v>26</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KZJ</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>